<commit_message>
add drag and drop question type (text-based over image); added preview item button
</commit_message>
<xml_diff>
--- a/examples/template.xlsx
+++ b/examples/template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Settings" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Questions" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A40"/>
+  <dimension ref="A1:A45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="118" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">                     true_false, single_checkbox, matching, sequence, numeric, short_answer.</t>
+          <t xml:space="preserve">                     true_false, single_checkbox, matching, sequence, numeric, short_answer, drag_drop.</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Scoring            Optional: all_or_nothing, partial, or weighted (choice/matching/sequence).</t>
+          <t xml:space="preserve">  Scoring            Optional: all_or_nothing, partial, or weighted (choice/matching/sequence/drag_drop).</t>
         </is>
       </c>
     </row>
@@ -756,10 +756,45 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr"/>
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  drag_drop (items into labeled boxes):</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Options = item=zone pairs separated by |  -&gt;  Router=Network | Switch=Data Link | Repeater=</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Zones are created in the order they first appear. Item=Zone A ; Zone B accepts either zone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Nothing after = makes a distractor (correct to leave unplaced). =Zone adds a zone with no correct item.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     Zone[n] limits a zone to n items, e.g. Router=Network[1]. Background-image zones need the builder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>TIP: The example rows already in the Questions sheet are a working quiz. Edit or delete them.</t>
         </is>
@@ -970,7 +1005,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1589,10 +1624,64 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr"/>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>drag_drop</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Drag each device onto the OSI layer where it primarily operates.</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>Map devices to OSI layers</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>OSI Model</t>
+        </is>
+      </c>
+      <c r="G12" s="8" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="H12" s="8" t="inlineStr">
+        <is>
+          <t>Router=Network | Switch=Data Link | Bridge=Data Link | Repeater=</t>
+        </is>
+      </c>
+      <c r="I12" s="8" t="inlineStr"/>
+      <c r="J12" s="8" t="inlineStr"/>
+      <c r="K12" s="8" t="inlineStr"/>
+      <c r="L12" s="8" t="inlineStr">
+        <is>
+          <t>Correct placement.</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="inlineStr">
+        <is>
+          <t>Check which address each device reads: IP or MAC.</t>
+        </is>
+      </c>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>Routers read IP (Layer 3); switches and bridges read MAC (Layer 2); a repeater is Layer 1.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"single_select,single_select_pill,multiple_select,multiple_select_pill,true_false,single_checkbox,matching,sequence,numeric,short_answer"</formula1>
+      <formula1>"single_select,single_select_pill,multiple_select,multiple_select_pill,true_false,single_checkbox,matching,sequence,numeric,short_answer,drag_drop"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>